<commit_message>
modificación del nombre de la tabla
</commit_message>
<xml_diff>
--- a/tabla final trabajo bootcamp.xlsx
+++ b/tabla final trabajo bootcamp.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bivi\Documents\GitHub\ProyectoAnalisisDeDatos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D672C332-BBC6-49AB-9067-3DE252351576}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C01252A-EA0C-4BB5-A775-056312ACD92F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{4CA48A38-0B0A-4ABF-95EE-D1684F7891C5}"/>
   </bookViews>
   <sheets>
-    <sheet name="tabla final trabajo bootcamp" sheetId="1" r:id="rId1"/>
+    <sheet name="Facturacion" sheetId="1" r:id="rId1"/>
     <sheet name="Pedido" sheetId="5" r:id="rId2"/>
     <sheet name="proveedor" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Facturacion!$A$1:$M$2031</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Pedido!$A$1:$H$1016</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">proveedor!$A$1:$D$1075</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'tabla final trabajo bootcamp'!$A$1:$M$2031</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>